<commit_message>
feat: add naver model v.6.4.1, v.6.4.2
</commit_message>
<xml_diff>
--- a/test_data/total_latest.xlsx
+++ b/test_data/total_latest.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I988"/>
+  <dimension ref="A1:I1008"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28643,10 +28643,10 @@
         <v>46265</v>
       </c>
       <c r="B973" t="n">
-        <v>15040</v>
+        <v>15034</v>
       </c>
       <c r="C973" t="n">
-        <v>4676</v>
+        <v>4674</v>
       </c>
       <c r="D973" t="n">
         <v>4016</v>
@@ -28658,13 +28658,13 @@
         <v>358</v>
       </c>
       <c r="G973" t="n">
-        <v>4991</v>
+        <v>4987</v>
       </c>
       <c r="H973" t="n">
-        <v>8692</v>
+        <v>8690</v>
       </c>
       <c r="I973" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="974">
@@ -28672,10 +28672,10 @@
         <v>46266</v>
       </c>
       <c r="B974" t="n">
-        <v>23435</v>
+        <v>23429</v>
       </c>
       <c r="C974" t="n">
-        <v>4616</v>
+        <v>4614</v>
       </c>
       <c r="D974" t="n">
         <v>4802</v>
@@ -28687,13 +28687,13 @@
         <v>516</v>
       </c>
       <c r="G974" t="n">
-        <v>12661</v>
+        <v>12657</v>
       </c>
       <c r="H974" t="n">
-        <v>9418</v>
+        <v>9416</v>
       </c>
       <c r="I974" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="975">
@@ -28701,10 +28701,10 @@
         <v>46267</v>
       </c>
       <c r="B975" t="n">
-        <v>22188</v>
+        <v>22182</v>
       </c>
       <c r="C975" t="n">
-        <v>5436</v>
+        <v>5434</v>
       </c>
       <c r="D975" t="n">
         <v>5620</v>
@@ -28716,13 +28716,13 @@
         <v>489</v>
       </c>
       <c r="G975" t="n">
-        <v>9855</v>
+        <v>9851</v>
       </c>
       <c r="H975" t="n">
-        <v>11056</v>
+        <v>11054</v>
       </c>
       <c r="I975" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="976">
@@ -28730,10 +28730,10 @@
         <v>46268</v>
       </c>
       <c r="B976" t="n">
-        <v>24353</v>
+        <v>24347</v>
       </c>
       <c r="C976" t="n">
-        <v>6222</v>
+        <v>6220</v>
       </c>
       <c r="D976" t="n">
         <v>6124</v>
@@ -28745,13 +28745,13 @@
         <v>503</v>
       </c>
       <c r="G976" t="n">
-        <v>10537</v>
+        <v>10533</v>
       </c>
       <c r="H976" t="n">
-        <v>12346</v>
+        <v>12344</v>
       </c>
       <c r="I976" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="977">
@@ -28759,10 +28759,10 @@
         <v>46269</v>
       </c>
       <c r="B977" t="n">
-        <v>23081</v>
+        <v>23075</v>
       </c>
       <c r="C977" t="n">
-        <v>6717</v>
+        <v>6715</v>
       </c>
       <c r="D977" t="n">
         <v>6191</v>
@@ -28774,13 +28774,13 @@
         <v>0</v>
       </c>
       <c r="G977" t="n">
-        <v>9305</v>
+        <v>9301</v>
       </c>
       <c r="H977" t="n">
-        <v>12908</v>
+        <v>12906</v>
       </c>
       <c r="I977" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="978">
@@ -28788,10 +28788,10 @@
         <v>46270</v>
       </c>
       <c r="B978" t="n">
-        <v>14893</v>
+        <v>14887</v>
       </c>
       <c r="C978" t="n">
-        <v>4304</v>
+        <v>4302</v>
       </c>
       <c r="D978" t="n">
         <v>3801</v>
@@ -28803,13 +28803,13 @@
         <v>160</v>
       </c>
       <c r="G978" t="n">
-        <v>6350</v>
+        <v>6346</v>
       </c>
       <c r="H978" t="n">
-        <v>8105</v>
+        <v>8103</v>
       </c>
       <c r="I978" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="979">
@@ -28817,10 +28817,10 @@
         <v>46271</v>
       </c>
       <c r="B979" t="n">
-        <v>18110</v>
+        <v>18104</v>
       </c>
       <c r="C979" t="n">
-        <v>4266</v>
+        <v>4264</v>
       </c>
       <c r="D979" t="n">
         <v>3461</v>
@@ -28832,13 +28832,13 @@
         <v>0</v>
       </c>
       <c r="G979" t="n">
-        <v>10243</v>
+        <v>10239</v>
       </c>
       <c r="H979" t="n">
-        <v>7727</v>
+        <v>7725</v>
       </c>
       <c r="I979" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="980">
@@ -28846,10 +28846,10 @@
         <v>46272</v>
       </c>
       <c r="B980" t="n">
-        <v>24020</v>
+        <v>24014</v>
       </c>
       <c r="C980" t="n">
-        <v>4856</v>
+        <v>4854</v>
       </c>
       <c r="D980" t="n">
         <v>4311</v>
@@ -28861,13 +28861,13 @@
         <v>1</v>
       </c>
       <c r="G980" t="n">
-        <v>13775</v>
+        <v>13771</v>
       </c>
       <c r="H980" t="n">
-        <v>9167</v>
+        <v>9165</v>
       </c>
       <c r="I980" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="981">
@@ -28875,10 +28875,10 @@
         <v>46273</v>
       </c>
       <c r="B981" t="n">
-        <v>23141</v>
+        <v>23134</v>
       </c>
       <c r="C981" t="n">
-        <v>5258</v>
+        <v>5256</v>
       </c>
       <c r="D981" t="n">
         <v>4820</v>
@@ -28890,13 +28890,13 @@
         <v>533</v>
       </c>
       <c r="G981" t="n">
-        <v>11573</v>
+        <v>11568</v>
       </c>
       <c r="H981" t="n">
-        <v>10078</v>
+        <v>10076</v>
       </c>
       <c r="I981" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="982">
@@ -28904,10 +28904,10 @@
         <v>46274</v>
       </c>
       <c r="B982" t="n">
-        <v>24372</v>
+        <v>24366</v>
       </c>
       <c r="C982" t="n">
-        <v>6070</v>
+        <v>6068</v>
       </c>
       <c r="D982" t="n">
         <v>5605</v>
@@ -28919,13 +28919,13 @@
         <v>534</v>
       </c>
       <c r="G982" t="n">
-        <v>11399</v>
+        <v>11395</v>
       </c>
       <c r="H982" t="n">
-        <v>11675</v>
+        <v>11673</v>
       </c>
       <c r="I982" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="983">
@@ -28933,10 +28933,10 @@
         <v>46275</v>
       </c>
       <c r="B983" t="n">
-        <v>32476</v>
+        <v>32470</v>
       </c>
       <c r="C983" t="n">
-        <v>7289</v>
+        <v>7287</v>
       </c>
       <c r="D983" t="n">
         <v>6989</v>
@@ -28948,13 +28948,13 @@
         <v>697</v>
       </c>
       <c r="G983" t="n">
-        <v>16523</v>
+        <v>16519</v>
       </c>
       <c r="H983" t="n">
-        <v>14278</v>
+        <v>14276</v>
       </c>
       <c r="I983" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="984">
@@ -28962,10 +28962,10 @@
         <v>46276</v>
       </c>
       <c r="B984" t="n">
-        <v>34448</v>
+        <v>34442</v>
       </c>
       <c r="C984" t="n">
-        <v>7511</v>
+        <v>7509</v>
       </c>
       <c r="D984" t="n">
         <v>8649</v>
@@ -28977,13 +28977,13 @@
         <v>767</v>
       </c>
       <c r="G984" t="n">
-        <v>16583</v>
+        <v>16579</v>
       </c>
       <c r="H984" t="n">
-        <v>16160</v>
+        <v>16158</v>
       </c>
       <c r="I984" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="985">
@@ -28991,10 +28991,10 @@
         <v>46277</v>
       </c>
       <c r="B985" t="n">
-        <v>21801</v>
+        <v>21795</v>
       </c>
       <c r="C985" t="n">
-        <v>4868</v>
+        <v>4866</v>
       </c>
       <c r="D985" t="n">
         <v>4383</v>
@@ -29006,13 +29006,13 @@
         <v>232</v>
       </c>
       <c r="G985" t="n">
-        <v>12105</v>
+        <v>12101</v>
       </c>
       <c r="H985" t="n">
-        <v>9251</v>
+        <v>9249</v>
       </c>
       <c r="I985" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="986">
@@ -29020,10 +29020,10 @@
         <v>46278</v>
       </c>
       <c r="B986" t="n">
-        <v>25161</v>
+        <v>25155</v>
       </c>
       <c r="C986" t="n">
-        <v>5116</v>
+        <v>5114</v>
       </c>
       <c r="D986" t="n">
         <v>3451</v>
@@ -29035,13 +29035,13 @@
         <v>0</v>
       </c>
       <c r="G986" t="n">
-        <v>16428</v>
+        <v>16424</v>
       </c>
       <c r="H986" t="n">
-        <v>8567</v>
+        <v>8565</v>
       </c>
       <c r="I986" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="987">
@@ -29049,10 +29049,10 @@
         <v>46279</v>
       </c>
       <c r="B987" t="n">
-        <v>32927</v>
+        <v>32921</v>
       </c>
       <c r="C987" t="n">
-        <v>6219</v>
+        <v>6217</v>
       </c>
       <c r="D987" t="n">
         <v>4491</v>
@@ -29064,13 +29064,13 @@
         <v>694</v>
       </c>
       <c r="G987" t="n">
-        <v>20314</v>
+        <v>20310</v>
       </c>
       <c r="H987" t="n">
-        <v>10710</v>
+        <v>10708</v>
       </c>
       <c r="I987" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="988">
@@ -29078,28 +29078,608 @@
         <v>46280</v>
       </c>
       <c r="B988" t="n">
-        <v>31376</v>
+        <v>31245</v>
       </c>
       <c r="C988" t="n">
-        <v>5914</v>
+        <v>5911</v>
       </c>
       <c r="D988" t="n">
-        <v>5447</v>
+        <v>5446</v>
       </c>
       <c r="E988" t="n">
-        <v>972</v>
+        <v>947</v>
       </c>
       <c r="F988" t="n">
         <v>488</v>
       </c>
       <c r="G988" t="n">
-        <v>18555</v>
+        <v>18453</v>
       </c>
       <c r="H988" t="n">
-        <v>11361</v>
+        <v>11357</v>
       </c>
       <c r="I988" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B989" t="n">
+        <v>32239</v>
+      </c>
+      <c r="C989" t="n">
+        <v>6539</v>
+      </c>
+      <c r="D989" t="n">
+        <v>6008</v>
+      </c>
+      <c r="E989" t="n">
+        <v>897</v>
+      </c>
+      <c r="F989" t="n">
+        <v>375</v>
+      </c>
+      <c r="G989" t="n">
+        <v>18420</v>
+      </c>
+      <c r="H989" t="n">
+        <v>12547</v>
+      </c>
+      <c r="I989" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B990" t="n">
+        <v>32321</v>
+      </c>
+      <c r="C990" t="n">
+        <v>7941</v>
+      </c>
+      <c r="D990" t="n">
+        <v>6805</v>
+      </c>
+      <c r="E990" t="n">
+        <v>969</v>
+      </c>
+      <c r="F990" t="n">
+        <v>392</v>
+      </c>
+      <c r="G990" t="n">
+        <v>16214</v>
+      </c>
+      <c r="H990" t="n">
+        <v>14746</v>
+      </c>
+      <c r="I990" t="n">
         <v>27</v>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B991" t="n">
+        <v>30284</v>
+      </c>
+      <c r="C991" t="n">
+        <v>7851</v>
+      </c>
+      <c r="D991" t="n">
+        <v>6582</v>
+      </c>
+      <c r="E991" t="n">
+        <v>785</v>
+      </c>
+      <c r="F991" t="n">
+        <v>301</v>
+      </c>
+      <c r="G991" t="n">
+        <v>14765</v>
+      </c>
+      <c r="H991" t="n">
+        <v>14433</v>
+      </c>
+      <c r="I991" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B992" t="n">
+        <v>17663</v>
+      </c>
+      <c r="C992" t="n">
+        <v>3699</v>
+      </c>
+      <c r="D992" t="n">
+        <v>4412</v>
+      </c>
+      <c r="E992" t="n">
+        <v>158</v>
+      </c>
+      <c r="F992" t="n">
+        <v>111</v>
+      </c>
+      <c r="G992" t="n">
+        <v>9283</v>
+      </c>
+      <c r="H992" t="n">
+        <v>8111</v>
+      </c>
+      <c r="I992" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B993" t="n">
+        <v>25237</v>
+      </c>
+      <c r="C993" t="n">
+        <v>5658</v>
+      </c>
+      <c r="D993" t="n">
+        <v>3710</v>
+      </c>
+      <c r="E993" t="n">
+        <v>171</v>
+      </c>
+      <c r="F993" t="n">
+        <v>0</v>
+      </c>
+      <c r="G993" t="n">
+        <v>15698</v>
+      </c>
+      <c r="H993" t="n">
+        <v>9368</v>
+      </c>
+      <c r="I993" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B994" t="n">
+        <v>33074</v>
+      </c>
+      <c r="C994" t="n">
+        <v>7254</v>
+      </c>
+      <c r="D994" t="n">
+        <v>5143</v>
+      </c>
+      <c r="E994" t="n">
+        <v>1181</v>
+      </c>
+      <c r="F994" t="n">
+        <v>305</v>
+      </c>
+      <c r="G994" t="n">
+        <v>19191</v>
+      </c>
+      <c r="H994" t="n">
+        <v>12397</v>
+      </c>
+      <c r="I994" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B995" t="n">
+        <v>31269</v>
+      </c>
+      <c r="C995" t="n">
+        <v>7455</v>
+      </c>
+      <c r="D995" t="n">
+        <v>6658</v>
+      </c>
+      <c r="E995" t="n">
+        <v>953</v>
+      </c>
+      <c r="F995" t="n">
+        <v>417</v>
+      </c>
+      <c r="G995" t="n">
+        <v>15786</v>
+      </c>
+      <c r="H995" t="n">
+        <v>14113</v>
+      </c>
+      <c r="I995" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B996" t="n">
+        <v>28359</v>
+      </c>
+      <c r="C996" t="n">
+        <v>8711</v>
+      </c>
+      <c r="D996" t="n">
+        <v>6571</v>
+      </c>
+      <c r="E996" t="n">
+        <v>1181</v>
+      </c>
+      <c r="F996" t="n">
+        <v>234</v>
+      </c>
+      <c r="G996" t="n">
+        <v>11662</v>
+      </c>
+      <c r="H996" t="n">
+        <v>15282</v>
+      </c>
+      <c r="I996" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B997" t="n">
+        <v>9284</v>
+      </c>
+      <c r="C997" t="n">
+        <v>16</v>
+      </c>
+      <c r="D997" t="n">
+        <v>11</v>
+      </c>
+      <c r="E997" t="n">
+        <v>7</v>
+      </c>
+      <c r="F997" t="n">
+        <v>0</v>
+      </c>
+      <c r="G997" t="n">
+        <v>9250</v>
+      </c>
+      <c r="H997" t="n">
+        <v>27</v>
+      </c>
+      <c r="I997" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B998" t="n">
+        <v>9122</v>
+      </c>
+      <c r="C998" t="n">
+        <v>13</v>
+      </c>
+      <c r="D998" t="n">
+        <v>4</v>
+      </c>
+      <c r="E998" t="n">
+        <v>3</v>
+      </c>
+      <c r="F998" t="n">
+        <v>1</v>
+      </c>
+      <c r="G998" t="n">
+        <v>9101</v>
+      </c>
+      <c r="H998" t="n">
+        <v>17</v>
+      </c>
+      <c r="I998" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B999" t="n">
+        <v>19933</v>
+      </c>
+      <c r="C999" t="n">
+        <v>5838</v>
+      </c>
+      <c r="D999" t="n">
+        <v>3064</v>
+      </c>
+      <c r="E999" t="n">
+        <v>134</v>
+      </c>
+      <c r="F999" t="n">
+        <v>0</v>
+      </c>
+      <c r="G999" t="n">
+        <v>10897</v>
+      </c>
+      <c r="H999" t="n">
+        <v>8902</v>
+      </c>
+      <c r="I999" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1000" t="n">
+        <v>31780</v>
+      </c>
+      <c r="C1000" t="n">
+        <v>7700</v>
+      </c>
+      <c r="D1000" t="n">
+        <v>4899</v>
+      </c>
+      <c r="E1000" t="n">
+        <v>1404</v>
+      </c>
+      <c r="F1000" t="n">
+        <v>688</v>
+      </c>
+      <c r="G1000" t="n">
+        <v>17089</v>
+      </c>
+      <c r="H1000" t="n">
+        <v>12599</v>
+      </c>
+      <c r="I1000" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1001" t="n">
+        <v>33845</v>
+      </c>
+      <c r="C1001" t="n">
+        <v>6910</v>
+      </c>
+      <c r="D1001" t="n">
+        <v>10955</v>
+      </c>
+      <c r="E1001" t="n">
+        <v>964</v>
+      </c>
+      <c r="F1001" t="n">
+        <v>346</v>
+      </c>
+      <c r="G1001" t="n">
+        <v>14670</v>
+      </c>
+      <c r="H1001" t="n">
+        <v>17865</v>
+      </c>
+      <c r="I1001" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B1002" t="n">
+        <v>29391</v>
+      </c>
+      <c r="C1002" t="n">
+        <v>4962</v>
+      </c>
+      <c r="D1002" t="n">
+        <v>9135</v>
+      </c>
+      <c r="E1002" t="n">
+        <v>735</v>
+      </c>
+      <c r="F1002" t="n">
+        <v>246</v>
+      </c>
+      <c r="G1002" t="n">
+        <v>14313</v>
+      </c>
+      <c r="H1002" t="n">
+        <v>14097</v>
+      </c>
+      <c r="I1002" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1003" t="n">
+        <v>39774</v>
+      </c>
+      <c r="C1003" t="n">
+        <v>7154</v>
+      </c>
+      <c r="D1003" t="n">
+        <v>12272</v>
+      </c>
+      <c r="E1003" t="n">
+        <v>945</v>
+      </c>
+      <c r="F1003" t="n">
+        <v>355</v>
+      </c>
+      <c r="G1003" t="n">
+        <v>19048</v>
+      </c>
+      <c r="H1003" t="n">
+        <v>19426</v>
+      </c>
+      <c r="I1003" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1004" t="n">
+        <v>36067</v>
+      </c>
+      <c r="C1004" t="n">
+        <v>7778</v>
+      </c>
+      <c r="D1004" t="n">
+        <v>11165</v>
+      </c>
+      <c r="E1004" t="n">
+        <v>700</v>
+      </c>
+      <c r="F1004" t="n">
+        <v>346</v>
+      </c>
+      <c r="G1004" t="n">
+        <v>16078</v>
+      </c>
+      <c r="H1004" t="n">
+        <v>18943</v>
+      </c>
+      <c r="I1004" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1005" t="n">
+        <v>25225</v>
+      </c>
+      <c r="C1005" t="n">
+        <v>6502</v>
+      </c>
+      <c r="D1005" t="n">
+        <v>5249</v>
+      </c>
+      <c r="E1005" t="n">
+        <v>132</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1005" t="n">
+        <v>13342</v>
+      </c>
+      <c r="H1005" t="n">
+        <v>11751</v>
+      </c>
+      <c r="I1005" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1006" t="n">
+        <v>30240</v>
+      </c>
+      <c r="C1006" t="n">
+        <v>5751</v>
+      </c>
+      <c r="D1006" t="n">
+        <v>8979</v>
+      </c>
+      <c r="E1006" t="n">
+        <v>153</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1006" t="n">
+        <v>15357</v>
+      </c>
+      <c r="H1006" t="n">
+        <v>14730</v>
+      </c>
+      <c r="I1006" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B1007" t="n">
+        <v>28097</v>
+      </c>
+      <c r="C1007" t="n">
+        <v>6344</v>
+      </c>
+      <c r="D1007" t="n">
+        <v>7963</v>
+      </c>
+      <c r="E1007" t="n">
+        <v>314</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1007" t="n">
+        <v>13476</v>
+      </c>
+      <c r="H1007" t="n">
+        <v>14307</v>
+      </c>
+      <c r="I1007" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1008" t="n">
+        <v>35585</v>
+      </c>
+      <c r="C1008" t="n">
+        <v>7556</v>
+      </c>
+      <c r="D1008" t="n">
+        <v>9509</v>
+      </c>
+      <c r="E1008" t="n">
+        <v>1622</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>612</v>
+      </c>
+      <c r="G1008" t="n">
+        <v>16286</v>
+      </c>
+      <c r="H1008" t="n">
+        <v>17065</v>
+      </c>
+      <c r="I1008" t="n">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>